<commit_message>
test: update dashboard test cases, rules, and executed evidence
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test-case-render/output/TestCase_Dashboard_Customer_retest_2026-10-18.xlsx
+++ b/test-case-render/output/TestCase_Dashboard_Customer_retest_2026-10-18.xlsx
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1965" uniqueCount="1030">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1992" uniqueCount="1030">
   <si>
     <t>Kết quả re-test dashboard Customer — ngày 18/10/2026</t>
   </si>
@@ -206,7 +206,7 @@
     <t>Kết quả mong đợi (Then)</t>
   </si>
   <si>
-    <t>passed/failed</t>
+    <t>20/10/2026</t>
   </si>
   <si>
     <t>Ghi chú</t>
@@ -215,7 +215,7 @@
     <t>Ưu tiên</t>
   </si>
   <si>
-    <t>Kết quả re-test 18/10/2026</t>
+    <t>18/10/2026</t>
   </si>
   <si>
     <t>Ghi chú re-test (thực tế quan sát trên https://ca-app.sts.vn/dashboard)</t>
@@ -3378,7 +3378,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="40">
+  <fills count="37">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -3448,24 +3448,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -3801,85 +3783,85 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -4214,7 +4196,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="304800"/>
+          <a:off x="24347170" y="3917315"/>
           <a:ext cx="5067300" cy="2660015"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4245,7 +4227,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="28599130" y="304800"/>
+          <a:off x="28599130" y="3917315"/>
           <a:ext cx="5067300" cy="2660015"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4276,7 +4258,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="304800"/>
+          <a:off x="24347170" y="3917315"/>
           <a:ext cx="5067300" cy="2660015"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4307,7 +4289,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="304800"/>
+          <a:off x="24347170" y="3917315"/>
           <a:ext cx="5067300" cy="2660015"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4338,7 +4320,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="28599130" y="304800"/>
+          <a:off x="28599130" y="3917315"/>
           <a:ext cx="5067300" cy="2542540"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4369,7 +4351,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="304800"/>
+          <a:off x="24347170" y="3917315"/>
           <a:ext cx="5067300" cy="2660015"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4400,7 +4382,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="28599130" y="304800"/>
+          <a:off x="28599130" y="3917315"/>
           <a:ext cx="5067300" cy="2660015"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4431,7 +4413,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="304800"/>
+          <a:off x="24347170" y="3917315"/>
           <a:ext cx="5067300" cy="2660015"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4462,7 +4444,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="304800"/>
+          <a:off x="24347170" y="3917315"/>
           <a:ext cx="5067300" cy="2660015"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4493,7 +4475,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="28599130" y="304800"/>
+          <a:off x="28599130" y="3917315"/>
           <a:ext cx="5067300" cy="2542540"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4524,7 +4506,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="304800"/>
+          <a:off x="24347170" y="3917315"/>
           <a:ext cx="5067300" cy="2660015"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4555,7 +4537,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="28599130" y="304800"/>
+          <a:off x="28599130" y="3917315"/>
           <a:ext cx="5067300" cy="2542540"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4586,7 +4568,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="304800"/>
+          <a:off x="24347170" y="3917315"/>
           <a:ext cx="5067300" cy="2660015"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4617,7 +4599,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="28599130" y="304800"/>
+          <a:off x="28599130" y="3917315"/>
           <a:ext cx="5067300" cy="2542540"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4648,7 +4630,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="1409700"/>
+          <a:off x="24347170" y="3917315"/>
           <a:ext cx="5067300" cy="2660015"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4679,7 +4661,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="28599130" y="1409700"/>
+          <a:off x="28599130" y="3917315"/>
           <a:ext cx="5067300" cy="2660015"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4710,7 +4692,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="1409700"/>
+          <a:off x="24347170" y="3917315"/>
           <a:ext cx="5067300" cy="2741295"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4741,7 +4723,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="4838700"/>
+          <a:off x="24347170" y="3917315"/>
           <a:ext cx="5067300" cy="1284605"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4772,7 +4754,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="6553200"/>
+          <a:off x="24347170" y="3917315"/>
           <a:ext cx="5067300" cy="1284605"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4803,7 +4785,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="8267700"/>
+          <a:off x="24347170" y="3917315"/>
           <a:ext cx="5067300" cy="2660015"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4834,7 +4816,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="8267700"/>
+          <a:off x="24347170" y="3917315"/>
           <a:ext cx="5067300" cy="2660015"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4865,7 +4847,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="28599130" y="8267700"/>
+          <a:off x="28599130" y="3917315"/>
           <a:ext cx="5067300" cy="2660015"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4896,7 +4878,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="8267700"/>
+          <a:off x="24347170" y="3917315"/>
           <a:ext cx="5067300" cy="2741295"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4927,7 +4909,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="8267700"/>
+          <a:off x="24347170" y="3917315"/>
           <a:ext cx="5067300" cy="2660015"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4958,7 +4940,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="8267700"/>
+          <a:off x="24347170" y="3917315"/>
           <a:ext cx="5067300" cy="2660015"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4989,7 +4971,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="8267700"/>
+          <a:off x="24347170" y="3917315"/>
           <a:ext cx="5067300" cy="2660015"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -5020,7 +5002,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="28599130" y="8267700"/>
+          <a:off x="28599130" y="3917315"/>
           <a:ext cx="5067300" cy="2660015"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -5051,7 +5033,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="8267700"/>
+          <a:off x="24347170" y="3917315"/>
           <a:ext cx="5067300" cy="2660015"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -5082,7 +5064,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="28599130" y="8267700"/>
+          <a:off x="28599130" y="3917315"/>
           <a:ext cx="5067300" cy="2660015"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -5113,7 +5095,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="8267700"/>
+          <a:off x="24347170" y="3917315"/>
           <a:ext cx="5067300" cy="2660015"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -5144,7 +5126,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="28599130" y="8267700"/>
+          <a:off x="28599130" y="3917315"/>
           <a:ext cx="5067300" cy="2578735"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -5175,7 +5157,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="17678400"/>
+          <a:off x="24347170" y="6679565"/>
           <a:ext cx="5067300" cy="2660015"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -5206,7 +5188,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="28599130" y="17678400"/>
+          <a:off x="28599130" y="6679565"/>
           <a:ext cx="5067300" cy="2578735"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -5237,7 +5219,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="20031075"/>
+          <a:off x="24347170" y="9441815"/>
           <a:ext cx="5067300" cy="2660015"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -5268,7 +5250,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="28599130" y="20031075"/>
+          <a:off x="28599130" y="9441815"/>
           <a:ext cx="5067300" cy="1130935"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -5299,7 +5281,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="36499800"/>
+          <a:off x="24347170" y="12204065"/>
           <a:ext cx="5067300" cy="2660015"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -5330,7 +5312,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="36499800"/>
+          <a:off x="24347170" y="12204065"/>
           <a:ext cx="5067300" cy="2578735"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -5361,7 +5343,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="36499800"/>
+          <a:off x="24347170" y="12204065"/>
           <a:ext cx="5067300" cy="2542540"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -5392,7 +5374,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="40119300"/>
+          <a:off x="24347170" y="12204065"/>
           <a:ext cx="5067300" cy="2542540"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -5423,7 +5405,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="28599130" y="40119300"/>
+          <a:off x="28599130" y="12204065"/>
           <a:ext cx="5067300" cy="2578735"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -5454,7 +5436,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="40119300"/>
+          <a:off x="24347170" y="12204065"/>
           <a:ext cx="5067300" cy="2542540"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -5485,7 +5467,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="40119300"/>
+          <a:off x="24347170" y="12204065"/>
           <a:ext cx="5067300" cy="1130935"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -5516,7 +5498,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="40119300"/>
+          <a:off x="24347170" y="14013815"/>
           <a:ext cx="5067300" cy="2578735"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -5547,7 +5529,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="40119300"/>
+          <a:off x="24347170" y="16694150"/>
           <a:ext cx="5067300" cy="1429385"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -5578,7 +5560,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="40119300"/>
+          <a:off x="24347170" y="16694150"/>
           <a:ext cx="5067300" cy="1130935"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -5609,7 +5591,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="40119300"/>
+          <a:off x="24347170" y="16694150"/>
           <a:ext cx="5067300" cy="2578735"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -5640,7 +5622,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="40119300"/>
+          <a:off x="24347170" y="16694150"/>
           <a:ext cx="5067300" cy="2578735"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -5671,7 +5653,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="28599130" y="40119300"/>
+          <a:off x="28599130" y="16694150"/>
           <a:ext cx="5067300" cy="2660015"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -5702,7 +5684,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="40119300"/>
+          <a:off x="24347170" y="19456400"/>
           <a:ext cx="5067300" cy="2578735"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -5733,7 +5715,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="40119300"/>
+          <a:off x="24347170" y="22136735"/>
           <a:ext cx="5067300" cy="2542540"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -5764,7 +5746,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="40119300"/>
+          <a:off x="24347170" y="22136735"/>
           <a:ext cx="5067300" cy="1429385"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -5795,7 +5777,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="40119300"/>
+          <a:off x="24347170" y="22136735"/>
           <a:ext cx="5067300" cy="2660015"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -5826,7 +5808,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="28599130" y="40119300"/>
+          <a:off x="28599130" y="22136735"/>
           <a:ext cx="5067300" cy="2542540"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -5857,7 +5839,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="41929050"/>
+          <a:off x="24347170" y="24898985"/>
           <a:ext cx="5067300" cy="1429385"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -5888,7 +5870,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="28599130" y="41929050"/>
+          <a:off x="28599130" y="24898985"/>
           <a:ext cx="5067300" cy="913765"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -5919,7 +5901,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="41929050"/>
+          <a:off x="24347170" y="24898985"/>
           <a:ext cx="5067300" cy="1492885"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -5950,7 +5932,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="41929050"/>
+          <a:off x="24347170" y="26642060"/>
           <a:ext cx="5067300" cy="1492885"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -5981,7 +5963,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="41929050"/>
+          <a:off x="24347170" y="28385135"/>
           <a:ext cx="5067300" cy="2660015"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -6012,7 +5994,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="28599130" y="41929050"/>
+          <a:off x="28599130" y="28385135"/>
           <a:ext cx="5067300" cy="2660015"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -6043,7 +6025,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="41929050"/>
+          <a:off x="24347170" y="28385135"/>
           <a:ext cx="5067300" cy="1492885"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -6074,7 +6056,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="41929050"/>
+          <a:off x="24347170" y="30128210"/>
           <a:ext cx="5067300" cy="1492885"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -6105,7 +6087,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="41929050"/>
+          <a:off x="24347170" y="30128210"/>
           <a:ext cx="5067300" cy="1492885"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -6136,7 +6118,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="28599130" y="41929050"/>
+          <a:off x="28599130" y="30128210"/>
           <a:ext cx="5067300" cy="2660015"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -6167,7 +6149,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="41929050"/>
+          <a:off x="24347170" y="30128210"/>
           <a:ext cx="5067300" cy="2741295"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -6198,7 +6180,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="28599130" y="41929050"/>
+          <a:off x="28599130" y="30128210"/>
           <a:ext cx="5067300" cy="2660015"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -6229,7 +6211,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="41929050"/>
+          <a:off x="24347170" y="30128210"/>
           <a:ext cx="5067300" cy="1492885"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -6260,7 +6242,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="41929050"/>
+          <a:off x="24347170" y="30128210"/>
           <a:ext cx="5067300" cy="913765"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -6291,7 +6273,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="28599130" y="41929050"/>
+          <a:off x="28599130" y="30128210"/>
           <a:ext cx="5067300" cy="1736725"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -6322,7 +6304,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="41929050"/>
+          <a:off x="24347170" y="30128210"/>
           <a:ext cx="5067300" cy="1736725"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -6353,7 +6335,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="28599130" y="41929050"/>
+          <a:off x="28599130" y="30128210"/>
           <a:ext cx="5067300" cy="1320800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -6384,7 +6366,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="41929050"/>
+          <a:off x="24347170" y="30128210"/>
           <a:ext cx="5067300" cy="913765"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -6415,7 +6397,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="28599130" y="41929050"/>
+          <a:off x="28599130" y="30128210"/>
           <a:ext cx="5067300" cy="1492885"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -6446,7 +6428,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="41929050"/>
+          <a:off x="24347170" y="30128210"/>
           <a:ext cx="5067300" cy="1529080"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -6477,7 +6459,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="41929050"/>
+          <a:off x="24347170" y="30128210"/>
           <a:ext cx="5067300" cy="1320800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -6508,7 +6490,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="28599130" y="41929050"/>
+          <a:off x="28599130" y="30128210"/>
           <a:ext cx="5067300" cy="2578735"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -6539,7 +6521,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="41929050"/>
+          <a:off x="24347170" y="32808545"/>
           <a:ext cx="5067300" cy="1736725"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -6570,7 +6552,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="28599130" y="41929050"/>
+          <a:off x="28599130" y="32808545"/>
           <a:ext cx="5067300" cy="1320800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -6601,7 +6583,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="41929050"/>
+          <a:off x="24347170" y="32808545"/>
           <a:ext cx="5067300" cy="1320800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -6632,7 +6614,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="41929050"/>
+          <a:off x="24347170" y="32808545"/>
           <a:ext cx="5067300" cy="1320800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -6663,7 +6645,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="51930300"/>
+          <a:off x="24347170" y="34808795"/>
           <a:ext cx="5067300" cy="1320800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -6694,7 +6676,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="28599130" y="51930300"/>
+          <a:off x="28599130" y="34808795"/>
           <a:ext cx="5067300" cy="2660015"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -6725,7 +6707,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="51930300"/>
+          <a:off x="24347170" y="37571045"/>
           <a:ext cx="5067300" cy="2660015"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -6756,7 +6738,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="51930300"/>
+          <a:off x="24347170" y="37571045"/>
           <a:ext cx="5067300" cy="2660015"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -6787,7 +6769,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="28599130" y="51930300"/>
+          <a:off x="28599130" y="37571045"/>
           <a:ext cx="5067300" cy="913765"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -6818,7 +6800,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="51930300"/>
+          <a:off x="24347170" y="37571045"/>
           <a:ext cx="5067300" cy="2660015"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -6849,7 +6831,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="28599130" y="51930300"/>
+          <a:off x="28599130" y="37571045"/>
           <a:ext cx="5067300" cy="1736725"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -6880,7 +6862,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="51930300"/>
+          <a:off x="24347170" y="37571045"/>
           <a:ext cx="5067300" cy="2542540"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -6911,7 +6893,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="28599130" y="51930300"/>
+          <a:off x="28599130" y="37571045"/>
           <a:ext cx="5067300" cy="2578735"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -6942,7 +6924,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="51930300"/>
+          <a:off x="24347170" y="37571045"/>
           <a:ext cx="5067300" cy="1492885"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -6973,7 +6955,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="51930300"/>
+          <a:off x="24347170" y="37571045"/>
           <a:ext cx="5067300" cy="2741295"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -7004,7 +6986,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="51930300"/>
+          <a:off x="24347170" y="37571045"/>
           <a:ext cx="5067300" cy="2660015"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -7035,7 +7017,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="51930300"/>
+          <a:off x="24347170" y="37571045"/>
           <a:ext cx="5067300" cy="2741295"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -7066,7 +7048,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="28599130" y="51930300"/>
+          <a:off x="28599130" y="37571045"/>
           <a:ext cx="5067300" cy="2162175"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -7097,7 +7079,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="51930300"/>
+          <a:off x="24347170" y="37571045"/>
           <a:ext cx="5067300" cy="1284605"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -7128,7 +7110,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="51930300"/>
+          <a:off x="24347170" y="37571045"/>
           <a:ext cx="5067300" cy="1691640"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -7159,7 +7141,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="28599130" y="51930300"/>
+          <a:off x="28599130" y="37571045"/>
           <a:ext cx="5067300" cy="1736725"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -7190,7 +7172,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="51930300"/>
+          <a:off x="24347170" y="37571045"/>
           <a:ext cx="5067300" cy="2162175"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -7221,7 +7203,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="51930300"/>
+          <a:off x="24347170" y="37571045"/>
           <a:ext cx="5067300" cy="2660015"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -7252,7 +7234,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="28599130" y="51930300"/>
+          <a:off x="28599130" y="37571045"/>
           <a:ext cx="5067300" cy="2660015"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -7283,7 +7265,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="51930300"/>
+          <a:off x="24347170" y="40333295"/>
           <a:ext cx="5067300" cy="1736725"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -7314,7 +7296,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="28599130" y="51930300"/>
+          <a:off x="28599130" y="40333295"/>
           <a:ext cx="5067300" cy="2660015"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -7345,7 +7327,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="51930300"/>
+          <a:off x="24347170" y="40333295"/>
           <a:ext cx="5067300" cy="1248410"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -7376,7 +7358,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="28599130" y="51930300"/>
+          <a:off x="28599130" y="40333295"/>
           <a:ext cx="5067300" cy="1736725"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -7407,7 +7389,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="51930300"/>
+          <a:off x="24347170" y="40333295"/>
           <a:ext cx="5067300" cy="2660015"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -7438,7 +7420,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="51930300"/>
+          <a:off x="24347170" y="40333295"/>
           <a:ext cx="5067300" cy="2660015"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -7469,7 +7451,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="51930300"/>
+          <a:off x="24347170" y="40333295"/>
           <a:ext cx="5067300" cy="2660015"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -7500,7 +7482,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="28599130" y="51930300"/>
+          <a:off x="28599130" y="40333295"/>
           <a:ext cx="5067300" cy="2660015"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -7531,7 +7513,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24347170" y="51930300"/>
+          <a:off x="24347170" y="40333295"/>
           <a:ext cx="5067300" cy="1691640"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -7562,7 +7544,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="28599130" y="51930300"/>
+          <a:off x="28599130" y="40333295"/>
           <a:ext cx="5067300" cy="1221105"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -8596,7 +8578,7 @@
       <c r="P10" s="6"/>
       <c r="Q10" s="6"/>
     </row>
-    <row r="11" ht="284.45" hidden="1" customHeight="1" spans="1:17">
+    <row r="11" ht="284.45" customHeight="1" spans="1:17">
       <c r="A11" s="4">
         <v>10</v>
       </c>
@@ -9282,7 +9264,7 @@
       <c r="P24" s="6"/>
       <c r="Q24" s="6"/>
     </row>
-    <row r="25" s="7" customFormat="1" ht="87" customHeight="1" spans="1:17">
+    <row r="25" s="7" customFormat="1" ht="87" hidden="1" customHeight="1" spans="1:17">
       <c r="A25" s="15">
         <v>24</v>
       </c>
@@ -9427,7 +9409,7 @@
       <c r="P27" s="6"/>
       <c r="Q27" s="6"/>
     </row>
-    <row r="28" ht="135" customHeight="1" spans="1:17">
+    <row r="28" ht="135" hidden="1" customHeight="1" spans="1:17">
       <c r="A28" s="4">
         <v>27</v>
       </c>
@@ -9455,7 +9437,9 @@
       <c r="I28" s="3" t="s">
         <v>268</v>
       </c>
-      <c r="J28" s="3"/>
+      <c r="J28" s="3" t="s">
+        <v>9</v>
+      </c>
       <c r="K28" s="3" t="s">
         <v>210</v>
       </c>
@@ -9466,7 +9450,7 @@
         <v>269</v>
       </c>
       <c r="N28" s="14" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="O28" s="10" t="s">
         <v>270</v>
@@ -9474,7 +9458,7 @@
       <c r="P28" s="6"/>
       <c r="Q28" s="6"/>
     </row>
-    <row r="29" ht="135" customHeight="1" spans="1:17">
+    <row r="29" ht="135" hidden="1" customHeight="1" spans="1:17">
       <c r="A29" s="4">
         <v>28</v>
       </c>
@@ -9502,7 +9486,9 @@
       <c r="I29" s="3" t="s">
         <v>274</v>
       </c>
-      <c r="J29" s="3"/>
+      <c r="J29" s="3" t="s">
+        <v>9</v>
+      </c>
       <c r="K29" s="3" t="s">
         <v>275</v>
       </c>
@@ -9513,7 +9499,7 @@
         <v>276</v>
       </c>
       <c r="N29" s="14" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="O29" s="10" t="s">
         <v>270</v>
@@ -9570,7 +9556,7 @@
       <c r="P30" s="6"/>
       <c r="Q30" s="6"/>
     </row>
-    <row r="31" s="7" customFormat="1" ht="135" customHeight="1" spans="1:17">
+    <row r="31" s="7" customFormat="1" ht="135" hidden="1" customHeight="1" spans="1:17">
       <c r="A31" s="15">
         <v>30</v>
       </c>
@@ -9666,7 +9652,7 @@
       <c r="P32" s="6"/>
       <c r="Q32" s="6"/>
     </row>
-    <row r="33" ht="135" customHeight="1" spans="1:17">
+    <row r="33" ht="135" hidden="1" customHeight="1" spans="1:17">
       <c r="A33" s="4">
         <v>32</v>
       </c>
@@ -9695,7 +9681,7 @@
         <v>299</v>
       </c>
       <c r="J33" s="3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="K33" s="3" t="s">
         <v>300</v>
@@ -10044,7 +10030,7 @@
       <c r="P40" s="6"/>
       <c r="Q40" s="6"/>
     </row>
-    <row r="41" ht="217.5" hidden="1" customHeight="1" spans="1:17">
+    <row r="41" ht="217.5" customHeight="1" spans="1:17">
       <c r="A41" s="4">
         <v>40</v>
       </c>
@@ -10072,7 +10058,9 @@
       <c r="I41" s="3" t="s">
         <v>357</v>
       </c>
-      <c r="J41" s="3"/>
+      <c r="J41" s="3" t="s">
+        <v>9</v>
+      </c>
       <c r="K41" s="3" t="s">
         <v>203</v>
       </c>
@@ -10140,7 +10128,7 @@
       <c r="P42" s="6"/>
       <c r="Q42" s="6"/>
     </row>
-    <row r="43" ht="185.25" customHeight="1" spans="1:17">
+    <row r="43" ht="185.25" hidden="1" customHeight="1" spans="1:17">
       <c r="A43" s="4">
         <v>42</v>
       </c>
@@ -10168,7 +10156,9 @@
       <c r="I43" s="3" t="s">
         <v>370</v>
       </c>
-      <c r="J43" s="3"/>
+      <c r="J43" s="3" t="s">
+        <v>9</v>
+      </c>
       <c r="K43" s="3" t="s">
         <v>371</v>
       </c>
@@ -10236,7 +10226,7 @@
       <c r="P44" s="6"/>
       <c r="Q44" s="6"/>
     </row>
-    <row r="45" ht="185.25" customHeight="1" spans="1:17">
+    <row r="45" ht="185.25" hidden="1" customHeight="1" spans="1:17">
       <c r="A45" s="4">
         <v>44</v>
       </c>
@@ -10264,7 +10254,9 @@
       <c r="I45" s="3" t="s">
         <v>382</v>
       </c>
-      <c r="J45" s="3"/>
+      <c r="J45" s="3" t="s">
+        <v>9</v>
+      </c>
       <c r="K45" s="3" t="s">
         <v>383</v>
       </c>
@@ -10283,7 +10275,7 @@
       <c r="P45" s="6"/>
       <c r="Q45" s="6"/>
     </row>
-    <row r="46" ht="185.25" customHeight="1" spans="1:17">
+    <row r="46" ht="185.25" hidden="1" customHeight="1" spans="1:17">
       <c r="A46" s="4">
         <v>45</v>
       </c>
@@ -10311,7 +10303,9 @@
       <c r="I46" s="3" t="s">
         <v>389</v>
       </c>
-      <c r="J46" s="3"/>
+      <c r="J46" s="3" t="s">
+        <v>9</v>
+      </c>
       <c r="K46" s="3" t="s">
         <v>383</v>
       </c>
@@ -10330,7 +10324,7 @@
       <c r="P46" s="6"/>
       <c r="Q46" s="6"/>
     </row>
-    <row r="47" ht="185.25" customHeight="1" spans="1:17">
+    <row r="47" ht="185.25" hidden="1" customHeight="1" spans="1:17">
       <c r="A47" s="4">
         <v>46</v>
       </c>
@@ -10358,7 +10352,9 @@
       <c r="I47" s="3" t="s">
         <v>394</v>
       </c>
-      <c r="J47" s="3"/>
+      <c r="J47" s="3" t="s">
+        <v>9</v>
+      </c>
       <c r="K47" s="3" t="s">
         <v>395</v>
       </c>
@@ -10377,7 +10373,7 @@
       <c r="P47" s="6"/>
       <c r="Q47" s="6"/>
     </row>
-    <row r="48" ht="217.5" hidden="1" customHeight="1" spans="1:17">
+    <row r="48" ht="217.5" customHeight="1" spans="1:17">
       <c r="A48" s="4">
         <v>47</v>
       </c>
@@ -10405,7 +10401,9 @@
       <c r="I48" s="3" t="s">
         <v>399</v>
       </c>
-      <c r="J48" s="3"/>
+      <c r="J48" s="3" t="s">
+        <v>9</v>
+      </c>
       <c r="K48" s="3" t="s">
         <v>400</v>
       </c>
@@ -10424,7 +10422,7 @@
       <c r="P48" s="6"/>
       <c r="Q48" s="6"/>
     </row>
-    <row r="49" ht="185.25" customHeight="1" spans="1:17">
+    <row r="49" ht="185.25" hidden="1" customHeight="1" spans="1:17">
       <c r="A49" s="4">
         <v>48</v>
       </c>
@@ -10452,7 +10450,9 @@
       <c r="I49" s="3" t="s">
         <v>405</v>
       </c>
-      <c r="J49" s="3"/>
+      <c r="J49" s="3" t="s">
+        <v>9</v>
+      </c>
       <c r="K49" s="3" t="s">
         <v>406</v>
       </c>
@@ -10471,7 +10471,7 @@
       <c r="P49" s="6"/>
       <c r="Q49" s="6"/>
     </row>
-    <row r="50" ht="217.5" hidden="1" customHeight="1" spans="1:17">
+    <row r="50" ht="217.5" customHeight="1" spans="1:17">
       <c r="A50" s="4">
         <v>49</v>
       </c>
@@ -10499,7 +10499,9 @@
       <c r="I50" s="3" t="s">
         <v>411</v>
       </c>
-      <c r="J50" s="3"/>
+      <c r="J50" s="3" t="s">
+        <v>9</v>
+      </c>
       <c r="K50" s="3" t="s">
         <v>412</v>
       </c>
@@ -10518,7 +10520,7 @@
       <c r="P50" s="6"/>
       <c r="Q50" s="6"/>
     </row>
-    <row r="51" ht="185.25" customHeight="1" spans="1:17">
+    <row r="51" ht="185.25" hidden="1" customHeight="1" spans="1:17">
       <c r="A51" s="4">
         <v>50</v>
       </c>
@@ -10546,7 +10548,9 @@
       <c r="I51" s="3" t="s">
         <v>418</v>
       </c>
-      <c r="J51" s="3"/>
+      <c r="J51" s="3" t="s">
+        <v>9</v>
+      </c>
       <c r="K51" s="3" t="s">
         <v>419</v>
       </c>
@@ -10565,7 +10569,7 @@
       <c r="P51" s="6"/>
       <c r="Q51" s="6"/>
     </row>
-    <row r="52" ht="185.25" customHeight="1" spans="1:17">
+    <row r="52" ht="185.25" hidden="1" customHeight="1" spans="1:17">
       <c r="A52" s="4">
         <v>51</v>
       </c>
@@ -10593,7 +10597,9 @@
       <c r="I52" s="3" t="s">
         <v>405</v>
       </c>
-      <c r="J52" s="3"/>
+      <c r="J52" s="3" t="s">
+        <v>9</v>
+      </c>
       <c r="K52" s="3" t="s">
         <v>425</v>
       </c>
@@ -10612,7 +10618,7 @@
       <c r="P52" s="6"/>
       <c r="Q52" s="6"/>
     </row>
-    <row r="53" ht="185.25" customHeight="1" spans="1:17">
+    <row r="53" ht="185.25" hidden="1" customHeight="1" spans="1:17">
       <c r="A53" s="4">
         <v>52</v>
       </c>
@@ -10640,7 +10646,9 @@
       <c r="I53" s="3" t="s">
         <v>430</v>
       </c>
-      <c r="J53" s="3"/>
+      <c r="J53" s="3" t="s">
+        <v>9</v>
+      </c>
       <c r="K53" s="3" t="s">
         <v>431</v>
       </c>
@@ -10659,7 +10667,7 @@
       <c r="P53" s="6"/>
       <c r="Q53" s="6"/>
     </row>
-    <row r="54" ht="185.25" customHeight="1" spans="1:17">
+    <row r="54" ht="185.25" hidden="1" customHeight="1" spans="1:17">
       <c r="A54" s="4">
         <v>53</v>
       </c>
@@ -10687,7 +10695,9 @@
       <c r="I54" s="3" t="s">
         <v>405</v>
       </c>
-      <c r="J54" s="3"/>
+      <c r="J54" s="3" t="s">
+        <v>9</v>
+      </c>
       <c r="K54" s="3" t="s">
         <v>436</v>
       </c>
@@ -10706,7 +10716,7 @@
       <c r="P54" s="6"/>
       <c r="Q54" s="6"/>
     </row>
-    <row r="55" ht="185.25" customHeight="1" spans="1:17">
+    <row r="55" ht="185.25" hidden="1" customHeight="1" spans="1:17">
       <c r="A55" s="4">
         <v>54</v>
       </c>
@@ -10753,7 +10763,7 @@
       <c r="P55" s="6"/>
       <c r="Q55" s="6"/>
     </row>
-    <row r="56" ht="185.25" customHeight="1" spans="1:17">
+    <row r="56" ht="185.25" hidden="1" customHeight="1" spans="1:17">
       <c r="A56" s="4">
         <v>55</v>
       </c>
@@ -10781,7 +10791,9 @@
       <c r="I56" s="3" t="s">
         <v>448</v>
       </c>
-      <c r="J56" s="3"/>
+      <c r="J56" s="3" t="s">
+        <v>9</v>
+      </c>
       <c r="K56" s="3" t="s">
         <v>449</v>
       </c>
@@ -10800,7 +10812,7 @@
       <c r="P56" s="6"/>
       <c r="Q56" s="6"/>
     </row>
-    <row r="57" ht="185.25" customHeight="1" spans="1:17">
+    <row r="57" ht="185.25" hidden="1" customHeight="1" spans="1:17">
       <c r="A57" s="4">
         <v>56</v>
       </c>
@@ -10990,7 +11002,7 @@
       <c r="P60" s="6"/>
       <c r="Q60" s="6"/>
     </row>
-    <row r="61" ht="142.5" customHeight="1" spans="1:17">
+    <row r="61" ht="142.5" hidden="1" customHeight="1" spans="1:17">
       <c r="A61" s="4">
         <v>60</v>
       </c>
@@ -11018,7 +11030,9 @@
       <c r="I61" s="3" t="s">
         <v>485</v>
       </c>
-      <c r="J61" s="3"/>
+      <c r="J61" s="3" t="s">
+        <v>9</v>
+      </c>
       <c r="K61" s="3" t="s">
         <v>486</v>
       </c>
@@ -11037,7 +11051,7 @@
       <c r="P61" s="6"/>
       <c r="Q61" s="6"/>
     </row>
-    <row r="62" ht="142.5" customHeight="1" spans="1:17">
+    <row r="62" ht="142.5" hidden="1" customHeight="1" spans="1:17">
       <c r="A62" s="4">
         <v>61</v>
       </c>
@@ -11065,7 +11079,9 @@
       <c r="I62" s="3" t="s">
         <v>492</v>
       </c>
-      <c r="J62" s="3"/>
+      <c r="J62" s="3" t="s">
+        <v>9</v>
+      </c>
       <c r="K62" s="3" t="s">
         <v>493</v>
       </c>
@@ -11178,7 +11194,7 @@
       <c r="P64" s="6"/>
       <c r="Q64" s="6"/>
     </row>
-    <row r="65" ht="142.5" hidden="1" customHeight="1" spans="1:17">
+    <row r="65" ht="142.5" customHeight="1" spans="1:17">
       <c r="A65" s="4">
         <v>64</v>
       </c>
@@ -11225,7 +11241,7 @@
       <c r="P65" s="6"/>
       <c r="Q65" s="6"/>
     </row>
-    <row r="66" ht="211.05" hidden="1" customHeight="1" spans="1:17">
+    <row r="66" ht="211.05" customHeight="1" spans="1:17">
       <c r="A66" s="4">
         <v>65</v>
       </c>
@@ -11253,7 +11269,9 @@
       <c r="I66" s="3" t="s">
         <v>516</v>
       </c>
-      <c r="J66" s="3"/>
+      <c r="J66" s="3" t="s">
+        <v>9</v>
+      </c>
       <c r="K66" s="3" t="s">
         <v>517</v>
       </c>
@@ -11464,7 +11482,7 @@
       <c r="P70" s="6"/>
       <c r="Q70" s="6"/>
     </row>
-    <row r="71" ht="217.5" hidden="1" customHeight="1" spans="1:17">
+    <row r="71" ht="217.5" customHeight="1" spans="1:17">
       <c r="A71" s="4">
         <v>70</v>
       </c>
@@ -11492,7 +11510,9 @@
       <c r="I71" s="3" t="s">
         <v>548</v>
       </c>
-      <c r="J71" s="3"/>
+      <c r="J71" s="3" t="s">
+        <v>9</v>
+      </c>
       <c r="K71" s="3" t="s">
         <v>549</v>
       </c>
@@ -11511,7 +11531,7 @@
       <c r="P71" s="6"/>
       <c r="Q71" s="6"/>
     </row>
-    <row r="72" ht="211.05" hidden="1" customHeight="1" spans="1:17">
+    <row r="72" ht="211.05" customHeight="1" spans="1:17">
       <c r="A72" s="4">
         <v>71</v>
       </c>
@@ -11539,7 +11559,9 @@
       <c r="I72" s="3" t="s">
         <v>553</v>
       </c>
-      <c r="J72" s="3"/>
+      <c r="J72" s="3" t="s">
+        <v>9</v>
+      </c>
       <c r="K72" s="3" t="s">
         <v>225</v>
       </c>
@@ -11795,7 +11817,7 @@
       <c r="P77" s="6"/>
       <c r="Q77" s="6"/>
     </row>
-    <row r="78" ht="217.5" hidden="1" customHeight="1" spans="1:17">
+    <row r="78" ht="217.5" customHeight="1" spans="1:17">
       <c r="A78" s="4">
         <v>77</v>
       </c>
@@ -11823,7 +11845,9 @@
       <c r="I78" s="3" t="s">
         <v>588</v>
       </c>
-      <c r="J78" s="3"/>
+      <c r="J78" s="3" t="s">
+        <v>9</v>
+      </c>
       <c r="K78" s="3" t="s">
         <v>589</v>
       </c>
@@ -11842,7 +11866,7 @@
       <c r="P78" s="6"/>
       <c r="Q78" s="6"/>
     </row>
-    <row r="79" ht="142.5" customHeight="1" spans="1:17">
+    <row r="79" ht="142.5" hidden="1" customHeight="1" spans="1:17">
       <c r="A79" s="4">
         <v>78</v>
       </c>
@@ -11871,7 +11895,7 @@
         <v>595</v>
       </c>
       <c r="J79" s="3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="K79" s="3" t="s">
         <v>596</v>
@@ -11938,7 +11962,7 @@
       <c r="P80" s="6"/>
       <c r="Q80" s="6"/>
     </row>
-    <row r="81" ht="137.25" hidden="1" customHeight="1" spans="1:17">
+    <row r="81" ht="137.25" customHeight="1" spans="1:17">
       <c r="A81" s="4">
         <v>80</v>
       </c>
@@ -11987,7 +12011,7 @@
       <c r="P81" s="6"/>
       <c r="Q81" s="6"/>
     </row>
-    <row r="82" s="7" customFormat="1" ht="137.25" hidden="1" customHeight="1" spans="1:17">
+    <row r="82" s="7" customFormat="1" ht="137.25" customHeight="1" spans="1:17">
       <c r="A82" s="15">
         <v>81</v>
       </c>
@@ -12015,7 +12039,9 @@
       <c r="I82" s="17" t="s">
         <v>618</v>
       </c>
-      <c r="J82" s="17"/>
+      <c r="J82" s="17" t="s">
+        <v>9</v>
+      </c>
       <c r="K82" s="17" t="s">
         <v>619</v>
       </c>
@@ -12132,7 +12158,7 @@
       <c r="P84" s="6"/>
       <c r="Q84" s="6"/>
     </row>
-    <row r="85" ht="137.25" hidden="1" customHeight="1" spans="1:17">
+    <row r="85" ht="137.25" customHeight="1" spans="1:17">
       <c r="A85" s="4">
         <v>84</v>
       </c>
@@ -13112,7 +13138,7 @@
       <c r="P104" s="6"/>
       <c r="Q104" s="6"/>
     </row>
-    <row r="105" ht="211.05" hidden="1" customHeight="1" spans="1:17">
+    <row r="105" ht="211.05" customHeight="1" spans="1:17">
       <c r="A105" s="4">
         <v>105</v>
       </c>
@@ -13351,7 +13377,7 @@
       <c r="P109" s="6"/>
       <c r="Q109" s="6"/>
     </row>
-    <row r="110" ht="157.5" hidden="1" customHeight="1" spans="1:17">
+    <row r="110" ht="157.5" customHeight="1" spans="1:17">
       <c r="A110" s="4">
         <v>110</v>
       </c>
@@ -13398,7 +13424,7 @@
       <c r="P110" s="6"/>
       <c r="Q110" s="6"/>
     </row>
-    <row r="111" ht="157.5" customHeight="1" spans="1:17">
+    <row r="111" ht="157.5" hidden="1" customHeight="1" spans="1:17">
       <c r="A111" s="4">
         <v>111</v>
       </c>
@@ -13426,7 +13452,9 @@
       <c r="I111" s="3" t="s">
         <v>804</v>
       </c>
-      <c r="J111" s="3"/>
+      <c r="J111" s="3" t="s">
+        <v>9</v>
+      </c>
       <c r="K111" s="3" t="s">
         <v>406</v>
       </c>
@@ -13445,7 +13473,7 @@
       <c r="P111" s="6"/>
       <c r="Q111" s="6"/>
     </row>
-    <row r="112" ht="157.5" customHeight="1" spans="1:17">
+    <row r="112" ht="157.5" hidden="1" customHeight="1" spans="1:17">
       <c r="A112" s="4">
         <v>112</v>
       </c>
@@ -13473,7 +13501,9 @@
       <c r="I112" s="3" t="s">
         <v>811</v>
       </c>
-      <c r="J112" s="3"/>
+      <c r="J112" s="3" t="s">
+        <v>9</v>
+      </c>
       <c r="K112" s="3" t="s">
         <v>578</v>
       </c>
@@ -13492,7 +13522,7 @@
       <c r="P112" s="6"/>
       <c r="Q112" s="6"/>
     </row>
-    <row r="113" ht="157.5" customHeight="1" spans="1:17">
+    <row r="113" ht="157.5" hidden="1" customHeight="1" spans="1:17">
       <c r="A113" s="4">
         <v>113</v>
       </c>
@@ -13520,7 +13550,9 @@
       <c r="I113" s="3" t="s">
         <v>816</v>
       </c>
-      <c r="J113" s="3"/>
+      <c r="J113" s="3" t="s">
+        <v>9</v>
+      </c>
       <c r="K113" s="3" t="s">
         <v>817</v>
       </c>
@@ -13539,7 +13571,7 @@
       <c r="P113" s="6"/>
       <c r="Q113" s="6"/>
     </row>
-    <row r="114" ht="157.5" customHeight="1" spans="1:17">
+    <row r="114" ht="157.5" hidden="1" customHeight="1" spans="1:17">
       <c r="A114" s="4">
         <v>114</v>
       </c>
@@ -13567,7 +13599,9 @@
       <c r="I114" s="3" t="s">
         <v>822</v>
       </c>
-      <c r="J114" s="3"/>
+      <c r="J114" s="3" t="s">
+        <v>9</v>
+      </c>
       <c r="K114" s="3" t="s">
         <v>769</v>
       </c>
@@ -13586,7 +13620,7 @@
       <c r="P114" s="6"/>
       <c r="Q114" s="6"/>
     </row>
-    <row r="115" ht="157.5" customHeight="1" spans="1:17">
+    <row r="115" ht="157.5" hidden="1" customHeight="1" spans="1:17">
       <c r="A115" s="4">
         <v>115</v>
       </c>
@@ -13635,7 +13669,7 @@
       <c r="P115" s="6"/>
       <c r="Q115" s="6"/>
     </row>
-    <row r="116" ht="217.5" hidden="1" customHeight="1" spans="1:17">
+    <row r="116" ht="217.5" customHeight="1" spans="1:17">
       <c r="A116" s="4">
         <v>116</v>
       </c>
@@ -13663,7 +13697,9 @@
       <c r="I116" s="3" t="s">
         <v>832</v>
       </c>
-      <c r="J116" s="3"/>
+      <c r="J116" s="3" t="s">
+        <v>9</v>
+      </c>
       <c r="K116" s="3" t="s">
         <v>833</v>
       </c>
@@ -14270,7 +14306,7 @@
       <c r="P128" s="6"/>
       <c r="Q128" s="6"/>
     </row>
-    <row r="129" ht="217.5" hidden="1" customHeight="1" spans="1:17">
+    <row r="129" ht="217.5" customHeight="1" spans="1:17">
       <c r="A129" s="4">
         <v>129</v>
       </c>
@@ -14615,14 +14651,9 @@
     </row>
   </sheetData>
   <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:Q135" etc:filterBottomFollowUsedRange="0">
-    <filterColumn colId="9">
-      <filters blank="1">
-        <filter val="failed"/>
-      </filters>
-    </filterColumn>
     <filterColumn colId="13">
       <filters>
-        <filter val="blocked (không test được)"/>
+        <filter val="failed"/>
       </filters>
     </filterColumn>
     <extLst/>

</xml_diff>